<commit_message>
added weekday and time of day preferences for single pracownik
</commit_message>
<xml_diff>
--- a/grafiki/grafik_stany_2026_09.xlsx
+++ b/grafiki/grafik_stany_2026_09.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ7"/>
+  <dimension ref="A1:AR8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,195 +439,200 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Dni pracy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>01.09 (Wt)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>02.09 (Śr)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>03.09 (Cz)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>04.09 (Pt)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>05.09 (Sb)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>06.09 (Nd)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>07.09 (Pn)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>08.09 (Wt)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>09.09 (Śr)</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>10.09 (Cz)</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>11.09 (Pt)</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>12.09 (Sb)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>13.09 (Nd)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>14.09 (Pn)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>15.09 (Wt)</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>16.09 (Śr)</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>17.09 (Cz)</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>18.09 (Pt)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>19.09 (Sb)</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>20.09 (Nd)</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>21.09 (Pn)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>22.09 (Wt)</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>23.09 (Śr)</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>24.09 (Cz)</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>25.09 (Pt)</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>26.09 (Sb)</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>27.09 (Nd)</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>28.09 (Pn)</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>29.09 (Wt)</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>30.09 (Śr)</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Suma godz.</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Bilans (h)</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>UUW</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>L4</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -652,7 +657,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>5,6,11,12,13,14,15,16,17,18,19,20,21,22,23,24,27,28,29,30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -800,15 +805,17 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AI2" t="n">
-        <v>0</v>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
       </c>
       <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
         <v>-160</v>
       </c>
-      <c r="AK2" t="n">
-        <v>0</v>
-      </c>
       <c r="AL2" t="n">
         <v>0</v>
       </c>
@@ -825,6 +832,9 @@
         <v>0</v>
       </c>
       <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -847,7 +857,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -892,24 +902,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>X</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>P</t>
@@ -995,15 +1005,17 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AI3" t="n">
-        <v>0</v>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
       </c>
       <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
         <v>-160</v>
       </c>
-      <c r="AK3" t="n">
-        <v>0</v>
-      </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
@@ -1020,6 +1032,9 @@
         <v>0</v>
       </c>
       <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1042,7 +1057,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1067,27 +1082,27 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>P</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1190,31 +1205,36 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AI4" t="n">
-        <v>44</v>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
       </c>
       <c r="AJ4" t="n">
-        <v>-36</v>
+        <v>36</v>
       </c>
       <c r="AK4" t="n">
-        <v>3</v>
+        <v>-44</v>
       </c>
       <c r="AL4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP4" t="n">
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1237,7 +1257,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1267,19 +1287,19 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>P</t>
@@ -1385,21 +1405,23 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AI5" t="n">
-        <v>36</v>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
       </c>
       <c r="AJ5" t="n">
-        <v>-84</v>
+        <v>24</v>
       </c>
       <c r="AK5" t="n">
-        <v>1</v>
+        <v>-96</v>
       </c>
       <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
         <v>2</v>
       </c>
-      <c r="AM5" t="n">
-        <v>0</v>
-      </c>
       <c r="AN5" t="n">
         <v>0</v>
       </c>
@@ -1410,6 +1432,9 @@
         <v>0</v>
       </c>
       <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1432,7 +1457,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1497,17 +1522,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1580,14 +1605,16 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>0</v>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
       </c>
       <c r="AJ6" t="n">
-        <v>-160</v>
+        <v>24</v>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
+        <v>-136</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
@@ -1596,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1605,117 +1632,321 @@
         <v>0</v>
       </c>
       <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>maks</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sprytny</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5,6,16,23,28,29</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>-80</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>PODSUMOWANIE</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>24</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M8" t="n">
         <v>24</v>
       </c>
-      <c r="M7" t="n">
-        <v>24</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
+      <c r="N8" t="n">
+        <v>12</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
looking between mounths, preferences from days and shifts from csv file for every employee, recalculating hours for mounth based on number of days
</commit_message>
<xml_diff>
--- a/grafiki/grafik_stany_2026_09.xlsx
+++ b/grafiki/grafik_stany_2026_09.xlsx
@@ -653,11 +653,11 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5,6,11,12,13,14,15,16,17,18,19,20,21,22,23,24,27,28,29,30</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -814,7 +814,7 @@
         <v>0</v>
       </c>
       <c r="AK2" t="n">
-        <v>-160</v>
+        <v>-176</v>
       </c>
       <c r="AL2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -853,41 +853,41 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -907,17 +907,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>P</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>P</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>P</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1011,10 +1011,10 @@
         </is>
       </c>
       <c r="AJ3" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="AK3" t="n">
-        <v>-160</v>
+        <v>-144</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
@@ -1023,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="AN3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AO3" t="n">
         <v>0</v>
@@ -1035,7 +1035,7 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1053,11 +1053,11 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1092,17 +1092,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>P</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>P</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1117,57 +1117,57 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1211,19 +1211,19 @@
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="AK4" t="n">
-        <v>-44</v>
+        <v>-60</v>
       </c>
       <c r="AL4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1250,14 +1250,14 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>120</v>
+        <v>176</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1292,12 +1292,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1411,16 +1411,16 @@
         </is>
       </c>
       <c r="AJ5" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="n">
-        <v>-96</v>
+        <v>-176</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1450,14 +1450,14 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D6" t="n">
-        <v>160</v>
+        <v>88</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31</t>
+          <t>12:D,13:D,18:N,19:N,20:N,25:N,26:N,27:N</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1472,57 +1472,57 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>UUW</t>
+          <t>X</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1611,10 +1611,10 @@
         </is>
       </c>
       <c r="AJ6" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="AK6" t="n">
-        <v>-136</v>
+        <v>-48</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
@@ -1623,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="AN6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AO6" t="n">
         <v>0</v>
@@ -1635,7 +1635,7 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -1650,69 +1650,69 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>176</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5,6,16,23,28,29</t>
+          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>UUW</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1811,10 +1811,10 @@
         </is>
       </c>
       <c r="AJ7" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="AK7" t="n">
-        <v>-80</v>
+        <v>-104</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
         <v>0</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AO7" t="n">
         <v>0</v>
@@ -1835,7 +1835,7 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1867,13 +1867,13 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fixed day-night shifts disproportion, completing mounth work hours with shorter shifts
</commit_message>
<xml_diff>
--- a/grafiki/grafik_stany_2026_09.xlsx
+++ b/grafiki/grafik_stany_2026_09.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grafik" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Swieta" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -857,7 +858,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
+          <t>1:DN,2:N,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:N,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:N,28:DN,29:DN,30:DN,31:DN</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1057,7 +1058,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1:DN,2:DN,3:DN,4:DN,5:DN,6:DN,7:DN,8:DN,9:DN,10:DN,11:DN,12:DN,13:DN,14:DN,15:DN,16:DN,17:DN,18:DN,19:DN,20:DN,21:DN,22:DN,23:DN,24:DN,25:DN,26:DN,27:DN,28:DN,29:DN,30:DN,31:DN</t>
+          <t>1:N,2:DN,4:D,5:N,6:N,8:D,9:N,10:D,11:N,12:N,14:D,15:N,16:D,17:N,18:DN,21:N,22:D,23:N,24:DN,27:N,28:D,29:N,30:DN,31:N</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1457,7 +1458,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>12:D,13:D,18:N,19:N,20:N,25:N,26:N,27:N</t>
+          <t>1:N,2:N,3:N,4:N,5:DN,6:DN,7:N,8:N,9:N,10:N,11:N,12:DN,13:DN,14:N,15:N,16:N,17:N,18:N,19:DN,20:DN,21:N,22:N,23:N,24:N,25:N,26:DN,27:DN,28:N,29:N,30:N,31:N</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1951,4 +1952,25 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dni_swiateczne</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>